<commit_message>
Manuscript: descriptor perturbation numbers at the upgraded magnitudes; Source Data for Figs 2, 4-6 and ED Figs 7-10; Fig. 5 README; docx figure map
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/SourceData_Fig2.xlsx
+++ b/source_data/SourceData_Fig2.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -524,27 +524,31 @@
           <t>analysis/meoh_catalyst_level_2026_10_19/summary.json (cat_primary.comparison)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>second bar (cat., lab. X)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>b</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ammonia leader changes</t>
+          <t>STY leader changes catalyst against catalyst, each entry free to raise its conversion to 0.95 X_eq with catalyst amount (primary count), inert-limited loop</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>analysis/nh3_field_expansion_2026_10_12/nh3_1_2/runs/pooled_vf_screen/summary_printed.json (primary, variants.per_g_metal_leaderboard, variants.Ru_recovery_90pct; bootstrap_papers, regret_bins)</t>
+          <t>analysis/meoh_catalyst_level_2026_10_19/summary.json (conversion_raised.cost_f0.95.cat_primary); per group: groups_catalyst_level_conversion_raised.csv</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>bar height = fraction; hatched height = regret_gt5pct_groups / groups (primary only)</t>
+          <t>first bar (cat., X raised)</t>
         </is>
       </c>
     </row>
@@ -556,47 +560,47 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>what the mismatched comparisons differ by (primary)</t>
+          <t>ammonia leader changes</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>analysis/nh3_field_expansion_2026_10_12/nh3_1_2/runs/pooled_vf_screen/summary_printed.json (primary.mismatch_kinds); plant-winner metal from group_metrics_printed.csv (plant_winner_metal)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>analysis/nh3_field_expansion_2026_10_12/nh3_1_2/runs/pooled_vf_screen/summary_printed.json (primary, variants.per_g_metal_leaderboard, variants.Ru_recovery_90pct; bootstrap_papers, regret_bins)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>bar height = fraction; hatched height = regret_gt5pct_groups / groups (primary only)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>comparison group 10.1021/acscatal.5c05984 | 100 bar | H2/CO2 4 | 10 NL/g/h</t>
+          <t>what the mismatched comparisons differ by (primary)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>analysis/meoh_literature_inversion_2026_10_05/literature_candidates.csv</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>x = STY (g_MeOH g_cat-1 h-1); filled y = cost_recycled_opt_inlet (EUR/t, inert-limited loop; purge_recycled_opt_inlet, fraction of loop gas); open y = cost_recycled_opt (no limit); marker area ~ SCH4; leaders of the inert-limited loop</t>
-        </is>
-      </c>
+          <t>analysis/nh3_field_expansion_2026_10_12/nh3_1_2/runs/pooled_vf_screen/summary_printed.json (primary.mismatch_kinds); plant-winner metal from group_metrics_printed.csv (plant_winner_metal)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>d</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>comparison group 10.1126/sciadv.abi6012 | 40 bar | H2/CO2 3 | 24 NL/g/h</t>
+          <t>comparison group 10.1021/acscatal.5c05984 | 100 bar | H2/CO2 4 | 10 NL/g/h</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -606,27 +610,49 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>x = STY (g_MeOH g_cat-1 h-1); filled y = cost_recycled_opt_inlet (EUR/t, inert-limited loop; purge_recycled_opt_inlet, fraction of loop gas); open y = cost_recycled_opt (no limit); marker area ~ SCO; leaders of the inert-limited loop</t>
+          <t>x = STY (g_MeOH g_cat-1 h-1); filled y = cost_recycled_opt_inlet (EUR/t, inert-limited loop; purge_recycled_opt_inlet, fraction of loop gas); open y = cost_recycled_opt (no limit); marker area ~ SCH4; leaders of the inert-limited loop</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>comparison group 10.1126/sciadv.abi6012 | 40 bar | H2/CO2 3 | 24 NL/g/h</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>analysis/meoh_literature_inversion_2026_10_05/literature_candidates.csv</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>x = STY (g_MeOH g_cat-1 h-1); filled y = cost_recycled_opt_inlet (EUR/t, inert-limited loop; purge_recycled_opt_inlet, fraction of loop gas); open y = cost_recycled_opt (no limit); marker area ~ SCO; leaders of the inert-limited loop</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>f</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>comparison group 10.1002/aenm.201801772 | 400 C | 5 MPa | H2/N2 3 | 6.6e+04 mL/g/h</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>analysis/nh3_field_expansion_2026_10_12/nh3_1_2/runs/pooled_vf_screen/candidates_printed.csv</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>paper_rate in umol g_cat-1 h-1; regret of the rate leader 0.1376 (group_metrics_printed.csv)</t>
         </is>
@@ -709,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -893,12 +919,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>XS</t>
+          <t>X</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X·S</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -913,7 +939,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>XS</t>
+          <t>X</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -923,30 +949,30 @@
         <v>50</v>
       </c>
       <c r="H6" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6172839506172839</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J6" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="K6" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L6" t="n">
-        <v>0.3885738456859771</v>
+        <v>0.6139646532492606</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>SMeOH</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>S_MeOH</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -961,7 +987,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>SMeOH</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -971,45 +997,45 @@
         <v>50</v>
       </c>
       <c r="H7" t="n">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3703703703703703</v>
       </c>
       <c r="J7" t="n">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="K7" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="L7" t="n">
-        <v>0.6139646532492606</v>
+        <v>0.3376083189067868</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SMeOH</t>
+          <t>STY_no_limit</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>S_MeOH</t>
+          <t>STY</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>inert-limited (primary)</t>
+          <t>no inlet limit</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>cost_recycled_opt_inlet</t>
+          <t>cost_recycled_opt</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SMeOH</t>
+          <t>STY</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -1019,86 +1045,45 @@
         <v>50</v>
       </c>
       <c r="H8" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="I8" t="n">
-        <v>0.3703703703703703</v>
+        <v>0.308641975308642</v>
       </c>
       <c r="J8" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="K8" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="L8" t="n">
-        <v>0.3376083189067868</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>STY_no_limit</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>STY</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>no inlet limit</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>cost_recycled_opt</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>STY</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>81</v>
-      </c>
-      <c r="G9" t="n">
-        <v>50</v>
-      </c>
-      <c r="H9" t="n">
-        <v>25</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.308641975308642</v>
-      </c>
-      <c r="J9" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" t="n">
-        <v>15</v>
-      </c>
-      <c r="L9" t="n">
         <v>0.03543670951859796</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M8" t="n">
         <v>0.1690095116151454</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N8" t="n">
         <v>0.4459623458409864</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>STY leader changes catalyst against catalyst (each catalyst at its best measured point), inert-limited loop</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>STY leader changes catalyst against catalyst (each catalyst at its best measured point), inert-limited loop</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>source: analysis/meoh_catalyst_level_2026_10_19/summary.json (cat_primary.comparison)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>source: analysis/meoh_catalyst_level_2026_10_19/summary.json (cat_primary.comparison)</t>
+          <t>second bar (cat., lab. X)</t>
         </is>
       </c>
     </row>
@@ -1162,6 +1147,99 @@
       </c>
       <c r="B19" t="n">
         <v>0.5333561643835613</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>STY leader changes catalyst against catalyst, each entry free to raise its conversion to 0.95 X_eq with catalyst amount (primary count), inert-limited loop</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>source: analysis/meoh_catalyst_level_2026_10_19/summary.json (conversion_raised.cost_f0.95.cat_primary); per group: groups_catalyst_level_conversion_raised.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>first bar (cat., X raised)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>comparisons with at least two catalysts</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>leader is another catalyst</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>of which cost gap above 5 %</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CI95 low (paper bootstrap)</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.2205820039880359</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CI95 high (paper bootstrap)</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.459016393442623</v>
       </c>
     </row>
   </sheetData>

</xml_diff>